<commit_message>
Grade 2026-10-23 picks: 10 graded (5-5), performance report updated
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/performance_report.xlsx
+++ b/outputs/performance_report.xlsx
@@ -474,31 +474,31 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="C2" t="n">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="D2" t="n">
-        <v>0.46</v>
+        <v>0.464</v>
       </c>
       <c r="E2" t="n">
-        <v>1425.69</v>
+        <v>1444.86</v>
       </c>
       <c r="F2" t="n">
-        <v>-57.55</v>
+        <v>-49.92</v>
       </c>
       <c r="G2" t="n">
-        <v>-0.0404</v>
+        <v>-0.0346</v>
       </c>
       <c r="H2" t="n">
-        <v>0.543</v>
+        <v>0.542</v>
       </c>
       <c r="I2" t="n">
         <v>-0.0009</v>
       </c>
       <c r="J2" t="n">
-        <v>0.47</v>
+        <v>0.455</v>
       </c>
     </row>
   </sheetData>
@@ -574,31 +574,31 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C2" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D2" t="n">
-        <v>0.5</v>
+        <v>0.588</v>
       </c>
       <c r="E2" t="n">
-        <v>211</v>
+        <v>223.12</v>
       </c>
       <c r="F2" t="n">
-        <v>7.85</v>
+        <v>20.7</v>
       </c>
       <c r="G2" t="n">
-        <v>0.0372</v>
+        <v>0.09279999999999999</v>
       </c>
       <c r="H2" t="n">
         <v>0.51</v>
       </c>
       <c r="I2" t="n">
-        <v>0.0033</v>
+        <v>0.0059</v>
       </c>
       <c r="J2" t="n">
-        <v>0.571</v>
+        <v>0.588</v>
       </c>
     </row>
     <row r="3">
@@ -642,31 +642,31 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="C4" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D4" t="n">
-        <v>0.422</v>
+        <v>0.42</v>
       </c>
       <c r="E4" t="n">
-        <v>660.23</v>
+        <v>664.1900000000001</v>
       </c>
       <c r="F4" t="n">
-        <v>-68.41</v>
+        <v>-70.55</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.1036</v>
+        <v>-0.1062</v>
       </c>
       <c r="H4" t="n">
-        <v>0.553</v>
+        <v>0.551</v>
       </c>
       <c r="I4" t="n">
-        <v>-0.0061</v>
+        <v>-0.0067</v>
       </c>
       <c r="J4" t="n">
-        <v>0.378</v>
+        <v>0.34</v>
       </c>
     </row>
     <row r="5">
@@ -676,31 +676,31 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C5" t="n">
         <v>12</v>
       </c>
       <c r="D5" t="n">
-        <v>0.571</v>
+        <v>0.545</v>
       </c>
       <c r="E5" t="n">
-        <v>315.21</v>
+        <v>317.62</v>
       </c>
       <c r="F5" t="n">
-        <v>14.74</v>
+        <v>12.33</v>
       </c>
       <c r="G5" t="n">
-        <v>0.0468</v>
+        <v>0.0388</v>
       </c>
       <c r="H5" t="n">
-        <v>0.5590000000000001</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="I5" t="n">
-        <v>-0.008</v>
+        <v>-0.008200000000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>0.333</v>
+        <v>0.318</v>
       </c>
     </row>
     <row r="6">
@@ -710,31 +710,31 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C6" t="n">
         <v>5</v>
       </c>
       <c r="D6" t="n">
-        <v>0.357</v>
+        <v>0.333</v>
       </c>
       <c r="E6" t="n">
-        <v>154.12</v>
+        <v>154.8</v>
       </c>
       <c r="F6" t="n">
-        <v>-26.54</v>
+        <v>-27.22</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.1722</v>
+        <v>-0.1758</v>
       </c>
       <c r="H6" t="n">
-        <v>0.527</v>
+        <v>0.528</v>
       </c>
       <c r="I6" t="n">
-        <v>0.0127</v>
+        <v>0.0123</v>
       </c>
       <c r="J6" t="n">
-        <v>0.786</v>
+        <v>0.8</v>
       </c>
     </row>
   </sheetData>
@@ -810,31 +810,31 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C2" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D2" t="n">
-        <v>0.455</v>
+        <v>0.444</v>
       </c>
       <c r="E2" t="n">
-        <v>941.6</v>
+        <v>947.97</v>
       </c>
       <c r="F2" t="n">
-        <v>-48.96</v>
+        <v>-53.5</v>
       </c>
       <c r="G2" t="n">
-        <v>-0.052</v>
+        <v>-0.0564</v>
       </c>
       <c r="H2" t="n">
         <v>0.539</v>
       </c>
       <c r="I2" t="n">
-        <v>-0.0062</v>
+        <v>-0.0068</v>
       </c>
       <c r="J2" t="n">
-        <v>0.379</v>
+        <v>0.347</v>
       </c>
     </row>
     <row r="3">
@@ -844,31 +844,31 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="C3" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="D3" t="n">
-        <v>0.471</v>
+        <v>0.5</v>
       </c>
       <c r="E3" t="n">
-        <v>484.09</v>
+        <v>496.89</v>
       </c>
       <c r="F3" t="n">
-        <v>-8.59</v>
+        <v>3.58</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.0177</v>
+        <v>0.0072</v>
       </c>
       <c r="H3" t="n">
-        <v>0.552</v>
+        <v>0.548</v>
       </c>
       <c r="I3" t="n">
-        <v>0.0092</v>
+        <v>0.009900000000000001</v>
       </c>
       <c r="J3" t="n">
-        <v>0.647</v>
+        <v>0.658</v>
       </c>
     </row>
   </sheetData>
@@ -919,16 +919,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C2" t="n">
-        <v>0.479</v>
+        <v>0.482</v>
       </c>
       <c r="D2" t="n">
-        <v>0.35</v>
+        <v>0.375</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.129</v>
+        <v>-0.107</v>
       </c>
     </row>
     <row r="3">
@@ -938,16 +938,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C3" t="n">
         <v>0.537</v>
       </c>
       <c r="D3" t="n">
-        <v>0.5620000000000001</v>
+        <v>0.5590000000000001</v>
       </c>
       <c r="E3" t="n">
-        <v>0.025</v>
+        <v>0.022</v>
       </c>
     </row>
     <row r="4">
@@ -957,16 +957,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C4" t="n">
         <v>0.5610000000000001</v>
       </c>
       <c r="D4" t="n">
-        <v>0.455</v>
+        <v>0.472</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.106</v>
+        <v>-0.089</v>
       </c>
     </row>
     <row r="5">
@@ -976,16 +976,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C5" t="n">
-        <v>0.594</v>
+        <v>0.593</v>
       </c>
       <c r="D5" t="n">
-        <v>0.308</v>
+        <v>0.286</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.286</v>
+        <v>-0.307</v>
       </c>
     </row>
     <row r="6">
@@ -1037,7 +1037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD101"/>
+  <dimension ref="A1:AF111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1191,6 +1191,16 @@
           <t>inj_note</t>
         </is>
       </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>tier</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>abs_spread</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1309,6 +1319,8 @@
           <t xml:space="preserve">Jusuf Nurkic out; Tony Bradley out; Trey Alexander out; </t>
         </is>
       </c>
+      <c r="AE2" t="inlineStr"/>
+      <c r="AF2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1427,6 +1439,8 @@
           <t xml:space="preserve">Jusuf Nurkic out; Tony Bradley out; Trey Alexander out; </t>
         </is>
       </c>
+      <c r="AE3" t="inlineStr"/>
+      <c r="AF3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1545,6 +1559,8 @@
           <t xml:space="preserve">Grant Williams out; Coby White out; Kon Knueppel out; </t>
         </is>
       </c>
+      <c r="AE4" t="inlineStr"/>
+      <c r="AF4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1661,6 +1677,8 @@
           <t xml:space="preserve">T.J. McConnell out; Aaron Nesmith out; Johnny Furphy out; </t>
         </is>
       </c>
+      <c r="AE5" t="inlineStr"/>
+      <c r="AF5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1777,6 +1795,8 @@
           <t xml:space="preserve">T.J. McConnell out; Aaron Nesmith out; Johnny Furphy out; </t>
         </is>
       </c>
+      <c r="AE6" t="inlineStr"/>
+      <c r="AF6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1895,6 +1915,8 @@
           <t xml:space="preserve">Grant Williams out; Coby White out; Kon Knueppel out; </t>
         </is>
       </c>
+      <c r="AE7" t="inlineStr"/>
+      <c r="AF7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2011,6 +2033,8 @@
           <t xml:space="preserve">Donte DiVincenzo out; </t>
         </is>
       </c>
+      <c r="AE8" t="inlineStr"/>
+      <c r="AF8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2125,6 +2149,8 @@
         <v>0</v>
       </c>
       <c r="AD9" t="inlineStr"/>
+      <c r="AE9" t="inlineStr"/>
+      <c r="AF9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2237,6 +2263,8 @@
         <v>0</v>
       </c>
       <c r="AD10" t="inlineStr"/>
+      <c r="AE10" t="inlineStr"/>
+      <c r="AF10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2355,6 +2383,8 @@
           <t xml:space="preserve">Grant Williams out; Coby White out; Kon Knueppel out; </t>
         </is>
       </c>
+      <c r="AE11" t="inlineStr"/>
+      <c r="AF11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2469,6 +2499,8 @@
         <v>0</v>
       </c>
       <c r="AD12" t="inlineStr"/>
+      <c r="AE12" t="inlineStr"/>
+      <c r="AF12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2581,6 +2613,8 @@
         <v>0</v>
       </c>
       <c r="AD13" t="inlineStr"/>
+      <c r="AE13" t="inlineStr"/>
+      <c r="AF13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2697,6 +2731,8 @@
           <t xml:space="preserve">Branden Carlson out; Shaedon Sharpe out; </t>
         </is>
       </c>
+      <c r="AE14" t="inlineStr"/>
+      <c r="AF14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2813,6 +2849,8 @@
           <t xml:space="preserve">Jimmy Butler III out; Kristaps Porzingis out; Moses Moody out; Brandin Podziemski out; </t>
         </is>
       </c>
+      <c r="AE15" t="inlineStr"/>
+      <c r="AF15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2931,6 +2969,8 @@
           <t xml:space="preserve">Dylan Cardwell out; Maxime Raynaud out; </t>
         </is>
       </c>
+      <c r="AE16" t="inlineStr"/>
+      <c r="AF16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3049,6 +3089,8 @@
           <t xml:space="preserve">Grant Williams out; Coby White out; Kon Knueppel out; </t>
         </is>
       </c>
+      <c r="AE17" t="inlineStr"/>
+      <c r="AF17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3167,6 +3209,8 @@
           <t xml:space="preserve">T.J. McConnell out; Aaron Nesmith out; Johnny Furphy out; </t>
         </is>
       </c>
+      <c r="AE18" t="inlineStr"/>
+      <c r="AF18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3285,6 +3329,8 @@
           <t xml:space="preserve">Donte DiVincenzo out; </t>
         </is>
       </c>
+      <c r="AE19" t="inlineStr"/>
+      <c r="AF19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3397,6 +3443,8 @@
           <t xml:space="preserve">Grant Williams out; Coby White out; Kon Knueppel out; </t>
         </is>
       </c>
+      <c r="AE20" t="inlineStr"/>
+      <c r="AF20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3515,6 +3563,8 @@
           <t xml:space="preserve">Nic Claxton out; Jordan Hawkins out; </t>
         </is>
       </c>
+      <c r="AE21" t="inlineStr"/>
+      <c r="AF21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3633,6 +3683,8 @@
           <t xml:space="preserve">Dylan Cardwell out; Maxime Raynaud out; </t>
         </is>
       </c>
+      <c r="AE22" t="inlineStr"/>
+      <c r="AF22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3747,6 +3799,8 @@
         <v>0</v>
       </c>
       <c r="AD23" t="inlineStr"/>
+      <c r="AE23" t="inlineStr"/>
+      <c r="AF23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3861,6 +3915,8 @@
         <v>0</v>
       </c>
       <c r="AD24" t="inlineStr"/>
+      <c r="AE24" t="inlineStr"/>
+      <c r="AF24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3975,6 +4031,8 @@
         <v>0</v>
       </c>
       <c r="AD25" t="inlineStr"/>
+      <c r="AE25" t="inlineStr"/>
+      <c r="AF25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -4091,6 +4149,8 @@
           <t xml:space="preserve">Grant Williams out; Coby White out; Kon Knueppel out; </t>
         </is>
       </c>
+      <c r="AE26" t="inlineStr"/>
+      <c r="AF26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -4209,6 +4269,8 @@
           <t xml:space="preserve">T.J. McConnell out; Aaron Nesmith out; Johnny Furphy out; </t>
         </is>
       </c>
+      <c r="AE27" t="inlineStr"/>
+      <c r="AF27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -4327,6 +4389,8 @@
           <t xml:space="preserve">Mouhamed Gueye out; </t>
         </is>
       </c>
+      <c r="AE28" t="inlineStr"/>
+      <c r="AF28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -4443,6 +4507,8 @@
           <t xml:space="preserve">Brandon Ingram out; Max Strus out; Jordan Miller out; Yanic Konan Niederhauser out; </t>
         </is>
       </c>
+      <c r="AE29" t="inlineStr"/>
+      <c r="AF29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -4557,6 +4623,8 @@
         <v>0</v>
       </c>
       <c r="AD30" t="inlineStr"/>
+      <c r="AE30" t="inlineStr"/>
+      <c r="AF30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -4675,6 +4743,8 @@
           <t xml:space="preserve">Jonathan Isaac out; Anthony Black out; Noah Penda out; </t>
         </is>
       </c>
+      <c r="AE31" t="inlineStr"/>
+      <c r="AF31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -4791,6 +4861,8 @@
           <t xml:space="preserve">T.J. McConnell out; Aaron Nesmith out; Johnny Furphy out; </t>
         </is>
       </c>
+      <c r="AE32" t="inlineStr"/>
+      <c r="AF32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -4909,6 +4981,8 @@
           <t xml:space="preserve">Brandon Ingram out; Max Strus out; Jordan Miller out; Yanic Konan Niederhauser out; </t>
         </is>
       </c>
+      <c r="AE33" t="inlineStr"/>
+      <c r="AF33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -5027,6 +5101,8 @@
           <t xml:space="preserve">Caleb Martin out; Santi Aldama out; </t>
         </is>
       </c>
+      <c r="AE34" t="inlineStr"/>
+      <c r="AF34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -5143,6 +5219,8 @@
           <t xml:space="preserve">Dylan Cardwell out; Maxime Raynaud out; </t>
         </is>
       </c>
+      <c r="AE35" t="inlineStr"/>
+      <c r="AF35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -5255,6 +5333,8 @@
         <v>0</v>
       </c>
       <c r="AD36" t="inlineStr"/>
+      <c r="AE36" t="inlineStr"/>
+      <c r="AF36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -5367,6 +5447,8 @@
           <t xml:space="preserve">Nic Claxton out; Jordan Hawkins out; </t>
         </is>
       </c>
+      <c r="AE37" t="inlineStr"/>
+      <c r="AF37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -5479,6 +5561,8 @@
         <v>0</v>
       </c>
       <c r="AD38" t="inlineStr"/>
+      <c r="AE38" t="inlineStr"/>
+      <c r="AF38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -5597,6 +5681,8 @@
           <t xml:space="preserve">Dylan Cardwell out; Maxime Raynaud out; </t>
         </is>
       </c>
+      <c r="AE39" t="inlineStr"/>
+      <c r="AF39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -5711,6 +5797,8 @@
         <v>0</v>
       </c>
       <c r="AD40" t="inlineStr"/>
+      <c r="AE40" t="inlineStr"/>
+      <c r="AF40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -5829,6 +5917,8 @@
           <t xml:space="preserve">Jimmy Butler III out; Kristaps Porzingis out; Moses Moody out; Brandin Podziemski out; </t>
         </is>
       </c>
+      <c r="AE41" t="inlineStr"/>
+      <c r="AF41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -5947,6 +6037,8 @@
           <t xml:space="preserve">Jonathan Isaac out; Anthony Black out; Noah Penda out; </t>
         </is>
       </c>
+      <c r="AE42" t="inlineStr"/>
+      <c r="AF42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -6061,6 +6153,8 @@
         <v>0</v>
       </c>
       <c r="AD43" t="inlineStr"/>
+      <c r="AE43" t="inlineStr"/>
+      <c r="AF43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -6179,6 +6273,8 @@
           <t xml:space="preserve">Jonathan Isaac out; Anthony Black out; Noah Penda out; </t>
         </is>
       </c>
+      <c r="AE44" t="inlineStr"/>
+      <c r="AF44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -6297,6 +6393,8 @@
           <t xml:space="preserve">Brandon Ingram out; Max Strus out; Jordan Miller out; Yanic Konan Niederhauser out; </t>
         </is>
       </c>
+      <c r="AE45" t="inlineStr"/>
+      <c r="AF45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -6413,6 +6511,8 @@
           <t xml:space="preserve">Caleb Martin out; Santi Aldama out; </t>
         </is>
       </c>
+      <c r="AE46" t="inlineStr"/>
+      <c r="AF46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -6531,6 +6631,8 @@
           <t xml:space="preserve">T.J. McConnell out; Aaron Nesmith out; Johnny Furphy out; </t>
         </is>
       </c>
+      <c r="AE47" t="inlineStr"/>
+      <c r="AF47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -6649,6 +6751,8 @@
           <t xml:space="preserve">Jonathan Isaac out; Anthony Black out; Noah Penda out; </t>
         </is>
       </c>
+      <c r="AE48" t="inlineStr"/>
+      <c r="AF48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -6767,6 +6871,8 @@
           <t xml:space="preserve">Jusuf Nurkic out; Tony Bradley out; Trey Alexander out; </t>
         </is>
       </c>
+      <c r="AE49" t="inlineStr"/>
+      <c r="AF49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -6885,6 +6991,8 @@
           <t xml:space="preserve">Jamir Watkins out; Tristan Vukcevic out; </t>
         </is>
       </c>
+      <c r="AE50" t="inlineStr"/>
+      <c r="AF50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -7003,6 +7111,8 @@
           <t xml:space="preserve">Jamir Watkins out; Tristan Vukcevic out; </t>
         </is>
       </c>
+      <c r="AE51" t="inlineStr"/>
+      <c r="AF51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -7119,6 +7229,8 @@
           <t xml:space="preserve">Caleb Martin out; Santi Aldama out; </t>
         </is>
       </c>
+      <c r="AE52" t="inlineStr"/>
+      <c r="AF52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -7235,6 +7347,8 @@
           <t xml:space="preserve">Nic Claxton out; Jordan Hawkins out; </t>
         </is>
       </c>
+      <c r="AE53" t="inlineStr"/>
+      <c r="AF53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -7351,6 +7465,8 @@
           <t xml:space="preserve">Brandon Ingram out; Max Strus out; Jordan Miller out; Yanic Konan Niederhauser out; </t>
         </is>
       </c>
+      <c r="AE54" t="inlineStr"/>
+      <c r="AF54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -7467,6 +7583,8 @@
           <t xml:space="preserve">Grant Williams out; Coby White out; Kon Knueppel out; </t>
         </is>
       </c>
+      <c r="AE55" t="inlineStr"/>
+      <c r="AF55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -7585,6 +7703,8 @@
           <t xml:space="preserve">Mark Williams out; </t>
         </is>
       </c>
+      <c r="AE56" t="inlineStr"/>
+      <c r="AF56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -7697,6 +7817,8 @@
         <v>0</v>
       </c>
       <c r="AD57" t="inlineStr"/>
+      <c r="AE57" t="inlineStr"/>
+      <c r="AF57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -7815,6 +7937,8 @@
           <t xml:space="preserve">Mark Williams out; </t>
         </is>
       </c>
+      <c r="AE58" t="inlineStr"/>
+      <c r="AF58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -7933,6 +8057,8 @@
           <t xml:space="preserve">Mouhamed Gueye out; </t>
         </is>
       </c>
+      <c r="AE59" t="inlineStr"/>
+      <c r="AF59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -8049,6 +8175,8 @@
           <t xml:space="preserve">Jusuf Nurkic out; Tony Bradley out; Trey Alexander out; </t>
         </is>
       </c>
+      <c r="AE60" t="inlineStr"/>
+      <c r="AF60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -8163,6 +8291,8 @@
         <v>0</v>
       </c>
       <c r="AD61" t="inlineStr"/>
+      <c r="AE61" t="inlineStr"/>
+      <c r="AF61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -8277,6 +8407,8 @@
         <v>0</v>
       </c>
       <c r="AD62" t="inlineStr"/>
+      <c r="AE62" t="inlineStr"/>
+      <c r="AF62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -8391,6 +8523,8 @@
         <v>0</v>
       </c>
       <c r="AD63" t="inlineStr"/>
+      <c r="AE63" t="inlineStr"/>
+      <c r="AF63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -8505,6 +8639,8 @@
         <v>0</v>
       </c>
       <c r="AD64" t="inlineStr"/>
+      <c r="AE64" t="inlineStr"/>
+      <c r="AF64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -8619,6 +8755,8 @@
         <v>0</v>
       </c>
       <c r="AD65" t="inlineStr"/>
+      <c r="AE65" t="inlineStr"/>
+      <c r="AF65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -8737,6 +8875,8 @@
           <t xml:space="preserve">Mouhamed Gueye out; </t>
         </is>
       </c>
+      <c r="AE66" t="inlineStr"/>
+      <c r="AF66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -8855,6 +8995,8 @@
           <t xml:space="preserve">Branden Carlson out; Shaedon Sharpe out; </t>
         </is>
       </c>
+      <c r="AE67" t="inlineStr"/>
+      <c r="AF67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -8973,6 +9115,8 @@
           <t xml:space="preserve">Jimmy Butler III out; Kristaps Porzingis out; Moses Moody out; Brandin Podziemski out; </t>
         </is>
       </c>
+      <c r="AE68" t="inlineStr"/>
+      <c r="AF68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -9087,6 +9231,8 @@
         <v>0</v>
       </c>
       <c r="AD69" t="inlineStr"/>
+      <c r="AE69" t="inlineStr"/>
+      <c r="AF69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -9201,6 +9347,8 @@
         <v>0</v>
       </c>
       <c r="AD70" t="inlineStr"/>
+      <c r="AE70" t="inlineStr"/>
+      <c r="AF70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -9317,6 +9465,8 @@
           <t xml:space="preserve">Branden Carlson out; Shaedon Sharpe out; </t>
         </is>
       </c>
+      <c r="AE71" t="inlineStr"/>
+      <c r="AF71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -9435,6 +9585,8 @@
           <t xml:space="preserve">Brandon Ingram out; Max Strus out; Jordan Miller out; Yanic Konan Niederhauser out; </t>
         </is>
       </c>
+      <c r="AE72" t="inlineStr"/>
+      <c r="AF72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -9549,6 +9701,8 @@
         <v>0</v>
       </c>
       <c r="AD73" t="inlineStr"/>
+      <c r="AE73" t="inlineStr"/>
+      <c r="AF73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -9667,6 +9821,8 @@
           <t xml:space="preserve">Caleb Martin out; Santi Aldama out; </t>
         </is>
       </c>
+      <c r="AE74" t="inlineStr"/>
+      <c r="AF74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -9781,6 +9937,8 @@
         <v>0</v>
       </c>
       <c r="AD75" t="inlineStr"/>
+      <c r="AE75" t="inlineStr"/>
+      <c r="AF75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -9899,6 +10057,8 @@
           <t xml:space="preserve">Jonathan Isaac out; Anthony Black out; Noah Penda out; </t>
         </is>
       </c>
+      <c r="AE76" t="inlineStr"/>
+      <c r="AF76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -10017,6 +10177,8 @@
           <t xml:space="preserve">Jonathan Isaac out; Anthony Black out; Noah Penda out; </t>
         </is>
       </c>
+      <c r="AE77" t="inlineStr"/>
+      <c r="AF77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -10135,6 +10297,8 @@
           <t xml:space="preserve">Mark Williams out; </t>
         </is>
       </c>
+      <c r="AE78" t="inlineStr"/>
+      <c r="AF78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -10253,6 +10417,8 @@
           <t xml:space="preserve">Nic Claxton out; Jordan Hawkins out; </t>
         </is>
       </c>
+      <c r="AE79" t="inlineStr"/>
+      <c r="AF79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -10371,6 +10537,8 @@
           <t xml:space="preserve">Dylan Cardwell out; Maxime Raynaud out; </t>
         </is>
       </c>
+      <c r="AE80" t="inlineStr"/>
+      <c r="AF80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -10485,6 +10653,8 @@
         <v>0</v>
       </c>
       <c r="AD81" t="inlineStr"/>
+      <c r="AE81" t="inlineStr"/>
+      <c r="AF81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -10603,6 +10773,8 @@
           <t xml:space="preserve">Caleb Martin out; Santi Aldama out; </t>
         </is>
       </c>
+      <c r="AE82" t="inlineStr"/>
+      <c r="AF82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -10719,6 +10891,8 @@
           <t xml:space="preserve">Jusuf Nurkic out; Tony Bradley out; Trey Alexander out; </t>
         </is>
       </c>
+      <c r="AE83" t="inlineStr"/>
+      <c r="AF83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -10837,6 +11011,8 @@
           <t xml:space="preserve">Caleb Martin out; Santi Aldama out; </t>
         </is>
       </c>
+      <c r="AE84" t="inlineStr"/>
+      <c r="AF84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -10955,6 +11131,8 @@
           <t xml:space="preserve">Jamir Watkins out; Tristan Vukcevic out; </t>
         </is>
       </c>
+      <c r="AE85" t="inlineStr"/>
+      <c r="AF85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -11071,6 +11249,8 @@
           <t xml:space="preserve">Branden Carlson out; Shaedon Sharpe out; </t>
         </is>
       </c>
+      <c r="AE86" t="inlineStr"/>
+      <c r="AF86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -11189,6 +11369,8 @@
           <t xml:space="preserve">Mark Williams out; </t>
         </is>
       </c>
+      <c r="AE87" t="inlineStr"/>
+      <c r="AF87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -11305,6 +11487,8 @@
           <t xml:space="preserve">Brandon Ingram out; Max Strus out; Jordan Miller out; Yanic Konan Niederhauser out; </t>
         </is>
       </c>
+      <c r="AE88" t="inlineStr"/>
+      <c r="AF88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -11423,6 +11607,8 @@
           <t xml:space="preserve">Jonathan Isaac out; Anthony Black out; Noah Penda out; </t>
         </is>
       </c>
+      <c r="AE89" t="inlineStr"/>
+      <c r="AF89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -11537,6 +11723,8 @@
         <v>0</v>
       </c>
       <c r="AD90" t="inlineStr"/>
+      <c r="AE90" t="inlineStr"/>
+      <c r="AF90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -11655,6 +11843,8 @@
           <t xml:space="preserve">Mouhamed Gueye out; </t>
         </is>
       </c>
+      <c r="AE91" t="inlineStr"/>
+      <c r="AF91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -11769,6 +11959,8 @@
         <v>0</v>
       </c>
       <c r="AD92" t="inlineStr"/>
+      <c r="AE92" t="inlineStr"/>
+      <c r="AF92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -11883,6 +12075,8 @@
         <v>0</v>
       </c>
       <c r="AD93" t="inlineStr"/>
+      <c r="AE93" t="inlineStr"/>
+      <c r="AF93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -12001,6 +12195,8 @@
           <t xml:space="preserve">T.J. McConnell out; Aaron Nesmith out; Johnny Furphy out; </t>
         </is>
       </c>
+      <c r="AE94" t="inlineStr"/>
+      <c r="AF94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -12119,6 +12315,8 @@
           <t xml:space="preserve">Donte DiVincenzo out; </t>
         </is>
       </c>
+      <c r="AE95" t="inlineStr"/>
+      <c r="AF95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -12235,6 +12433,8 @@
           <t xml:space="preserve">Brandon Ingram out; Max Strus out; Jordan Miller out; Yanic Konan Niederhauser out; </t>
         </is>
       </c>
+      <c r="AE96" t="inlineStr"/>
+      <c r="AF96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -12351,6 +12551,8 @@
           <t xml:space="preserve">Nic Claxton out; Jordan Hawkins out; </t>
         </is>
       </c>
+      <c r="AE97" t="inlineStr"/>
+      <c r="AF97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -12469,6 +12671,8 @@
           <t xml:space="preserve">Jamir Watkins out; Tristan Vukcevic out; </t>
         </is>
       </c>
+      <c r="AE98" t="inlineStr"/>
+      <c r="AF98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -12585,6 +12789,8 @@
           <t xml:space="preserve">Grant Williams out; Coby White out; Kon Knueppel out; </t>
         </is>
       </c>
+      <c r="AE99" t="inlineStr"/>
+      <c r="AF99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -12699,6 +12905,8 @@
         <v>0</v>
       </c>
       <c r="AD100" t="inlineStr"/>
+      <c r="AE100" t="inlineStr"/>
+      <c r="AF100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -12814,6 +13022,1242 @@
         <is>
           <t xml:space="preserve">Brandon Ingram out; Max Strus out; Jordan Miller out; Yanic Konan Niederhauser out; </t>
         </is>
+      </c>
+      <c r="AE101" t="inlineStr"/>
+      <c r="AF101" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>NOP @ UTA</t>
+        </is>
+      </c>
+      <c r="C102" t="n">
+        <v>4066336</v>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Lauri Markkanen</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>lauri markkanen</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>UTA</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>NOP</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>PTS</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>over</t>
+        </is>
+      </c>
+      <c r="J102" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>betrivers</t>
+        </is>
+      </c>
+      <c r="L102" t="n">
+        <v>-129</v>
+      </c>
+      <c r="M102" t="n">
+        <v>26.84</v>
+      </c>
+      <c r="N102" t="n">
+        <v>0.8266</v>
+      </c>
+      <c r="O102" t="n">
+        <v>0.5317</v>
+      </c>
+      <c r="P102" t="n">
+        <v>0.5802</v>
+      </c>
+      <c r="Q102" t="n">
+        <v>0.0485</v>
+      </c>
+      <c r="R102" t="n">
+        <v>0.0299</v>
+      </c>
+      <c r="S102" t="n">
+        <v>2.41</v>
+      </c>
+      <c r="T102" t="inlineStr">
+        <is>
+          <t>7469a7f48dbb77001b3148829f80c97b</t>
+        </is>
+      </c>
+      <c r="U102" t="inlineStr">
+        <is>
+          <t>2026-10-23T12:45:33.160380+00:00</t>
+        </is>
+      </c>
+      <c r="V102" t="n">
+        <v>16</v>
+      </c>
+      <c r="W102" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="X102" t="n">
+        <v>-122</v>
+      </c>
+      <c r="Y102" t="n">
+        <v>0.5202</v>
+      </c>
+      <c r="Z102" t="n">
+        <v>-0.0115</v>
+      </c>
+      <c r="AA102" t="n">
+        <v>-2.41</v>
+      </c>
+      <c r="AB102" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC102" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jusuf Nurkic out; </t>
+        </is>
+      </c>
+      <c r="AE102" t="inlineStr">
+        <is>
+          <t>over (experimental) (early)</t>
+        </is>
+      </c>
+      <c r="AF102" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>NYK @ BOS</t>
+        </is>
+      </c>
+      <c r="C103" t="n">
+        <v>3136195</v>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Karl-Anthony Towns</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>karl anthony towns</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>NYK</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>BOS</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>AST</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>under</t>
+        </is>
+      </c>
+      <c r="J103" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>draftkings</t>
+        </is>
+      </c>
+      <c r="L103" t="n">
+        <v>122</v>
+      </c>
+      <c r="M103" t="n">
+        <v>2.67</v>
+      </c>
+      <c r="N103" t="n">
+        <v>0.7107</v>
+      </c>
+      <c r="O103" t="n">
+        <v>0.4278</v>
+      </c>
+      <c r="P103" t="n">
+        <v>0.4743</v>
+      </c>
+      <c r="Q103" t="n">
+        <v>0.0465</v>
+      </c>
+      <c r="R103" t="n">
+        <v>0.0528</v>
+      </c>
+      <c r="S103" t="n">
+        <v>5.42</v>
+      </c>
+      <c r="T103" t="inlineStr">
+        <is>
+          <t>0d34c898f6cbb990077ae9f0a2773513</t>
+        </is>
+      </c>
+      <c r="U103" t="inlineStr">
+        <is>
+          <t>2026-10-23T12:45:33.160380+00:00</t>
+        </is>
+      </c>
+      <c r="V103" t="n">
+        <v>3</v>
+      </c>
+      <c r="W103" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="X103" t="n">
+        <v>100</v>
+      </c>
+      <c r="Y103" t="n">
+        <v>0.4677</v>
+      </c>
+      <c r="Z103" t="n">
+        <v>0.0399</v>
+      </c>
+      <c r="AA103" t="n">
+        <v>6.612399999999998</v>
+      </c>
+      <c r="AB103" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC103" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD103" t="inlineStr"/>
+      <c r="AE103" t="inlineStr">
+        <is>
+          <t>core (early)</t>
+        </is>
+      </c>
+      <c r="AF103" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>NOP @ UTA</t>
+        </is>
+      </c>
+      <c r="C104" t="n">
+        <v>4066336</v>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Lauri Markkanen</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>lauri markkanen</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>UTA</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>NOP</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>PRA</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>over</t>
+        </is>
+      </c>
+      <c r="J104" t="n">
+        <v>31.5</v>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>fanduel</t>
+        </is>
+      </c>
+      <c r="L104" t="n">
+        <v>-118</v>
+      </c>
+      <c r="M104" t="n">
+        <v>36.26</v>
+      </c>
+      <c r="N104" t="n">
+        <v>0.7445000000000001</v>
+      </c>
+      <c r="O104" t="n">
+        <v>0.5122</v>
+      </c>
+      <c r="P104" t="n">
+        <v>0.5503</v>
+      </c>
+      <c r="Q104" t="n">
+        <v>0.0382</v>
+      </c>
+      <c r="R104" t="n">
+        <v>0.0167</v>
+      </c>
+      <c r="S104" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="T104" t="inlineStr">
+        <is>
+          <t>7469a7f48dbb77001b3148829f80c97b</t>
+        </is>
+      </c>
+      <c r="U104" t="inlineStr">
+        <is>
+          <t>2026-10-23T12:45:33.160380+00:00</t>
+        </is>
+      </c>
+      <c r="V104" t="n">
+        <v>25</v>
+      </c>
+      <c r="W104" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="X104" t="n">
+        <v>-118</v>
+      </c>
+      <c r="Y104" t="n">
+        <v>0.5101</v>
+      </c>
+      <c r="Z104" t="n">
+        <v>-0.0021</v>
+      </c>
+      <c r="AA104" t="n">
+        <v>-1.23</v>
+      </c>
+      <c r="AB104" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC104" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jusuf Nurkic out; </t>
+        </is>
+      </c>
+      <c r="AE104" t="inlineStr">
+        <is>
+          <t>over (experimental) (early)</t>
+        </is>
+      </c>
+      <c r="AF104" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>CHI @ MIL</t>
+        </is>
+      </c>
+      <c r="C105" t="n">
+        <v>5044385</v>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Leonard Miller</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>leonard miller</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>CHI</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>MIL</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>PRA</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>over</t>
+        </is>
+      </c>
+      <c r="J105" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>draftkings</t>
+        </is>
+      </c>
+      <c r="L105" t="n">
+        <v>-109</v>
+      </c>
+      <c r="M105" t="n">
+        <v>21.2</v>
+      </c>
+      <c r="N105" t="n">
+        <v>0.6988</v>
+      </c>
+      <c r="O105" t="n">
+        <v>0.4898</v>
+      </c>
+      <c r="P105" t="n">
+        <v>0.5241</v>
+      </c>
+      <c r="Q105" t="n">
+        <v>0.0343</v>
+      </c>
+      <c r="R105" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="S105" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="T105" t="inlineStr">
+        <is>
+          <t>0cdc865f5b785c0be6bc409117fe38aa</t>
+        </is>
+      </c>
+      <c r="U105" t="inlineStr">
+        <is>
+          <t>2026-10-23T12:45:33.160380+00:00</t>
+        </is>
+      </c>
+      <c r="V105" t="n">
+        <v>24</v>
+      </c>
+      <c r="W105" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="X105" t="n">
+        <v>-109</v>
+      </c>
+      <c r="Y105" t="n">
+        <v>0.4892</v>
+      </c>
+      <c r="Z105" t="n">
+        <v>-0.0005999999999999999</v>
+      </c>
+      <c r="AA105" t="n">
+        <v>0.3119266055045872</v>
+      </c>
+      <c r="AB105" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC105" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nic Claxton out; </t>
+        </is>
+      </c>
+      <c r="AE105" t="inlineStr">
+        <is>
+          <t>over (experimental) (early)</t>
+        </is>
+      </c>
+      <c r="AF105" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>NOP @ UTA</t>
+        </is>
+      </c>
+      <c r="C106" t="n">
+        <v>4395628</v>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Zion Williamson</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>zion williamson</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>NOP</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>UTA</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>PRA</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>over</t>
+        </is>
+      </c>
+      <c r="J106" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>fanduel</t>
+        </is>
+      </c>
+      <c r="L106" t="n">
+        <v>-120</v>
+      </c>
+      <c r="M106" t="n">
+        <v>31.12</v>
+      </c>
+      <c r="N106" t="n">
+        <v>0.7115</v>
+      </c>
+      <c r="O106" t="n">
+        <v>0.5184</v>
+      </c>
+      <c r="P106" t="n">
+        <v>0.5501</v>
+      </c>
+      <c r="Q106" t="n">
+        <v>0.0317</v>
+      </c>
+      <c r="R106" t="n">
+        <v>0.008500000000000001</v>
+      </c>
+      <c r="S106" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="T106" t="inlineStr">
+        <is>
+          <t>7469a7f48dbb77001b3148829f80c97b</t>
+        </is>
+      </c>
+      <c r="U106" t="inlineStr">
+        <is>
+          <t>2026-10-23T12:45:33.160380+00:00</t>
+        </is>
+      </c>
+      <c r="V106" t="n">
+        <v>30</v>
+      </c>
+      <c r="W106" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="X106" t="n">
+        <v>-118</v>
+      </c>
+      <c r="Y106" t="n">
+        <v>0.502</v>
+      </c>
+      <c r="Z106" t="n">
+        <v>-0.0164</v>
+      </c>
+      <c r="AA106" t="n">
+        <v>0.5333333333333334</v>
+      </c>
+      <c r="AB106" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC106" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD106" t="inlineStr"/>
+      <c r="AE106" t="inlineStr">
+        <is>
+          <t>over (experimental) (early)</t>
+        </is>
+      </c>
+      <c r="AF106" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>MEM @ GSW</t>
+        </is>
+      </c>
+      <c r="C107" t="n">
+        <v>3213</v>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Al Horford</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>al horford</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>GSW</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>MEM</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>PRA</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>over</t>
+        </is>
+      </c>
+      <c r="J107" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>fanduel</t>
+        </is>
+      </c>
+      <c r="L107" t="n">
+        <v>100</v>
+      </c>
+      <c r="M107" t="n">
+        <v>16.68</v>
+      </c>
+      <c r="N107" t="n">
+        <v>0.6735</v>
+      </c>
+      <c r="O107" t="n">
+        <v>0.4811</v>
+      </c>
+      <c r="P107" t="n">
+        <v>0.5127</v>
+      </c>
+      <c r="Q107" t="n">
+        <v>0.0316</v>
+      </c>
+      <c r="R107" t="n">
+        <v>0.0255</v>
+      </c>
+      <c r="S107" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="T107" t="inlineStr">
+        <is>
+          <t>d7525d3e92349ef234ca0c1ac699b365</t>
+        </is>
+      </c>
+      <c r="U107" t="inlineStr">
+        <is>
+          <t>2026-10-23T12:45:33.160380+00:00</t>
+        </is>
+      </c>
+      <c r="V107" t="n">
+        <v>8</v>
+      </c>
+      <c r="W107" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="X107" t="inlineStr"/>
+      <c r="Y107" t="n">
+        <v>0.4459</v>
+      </c>
+      <c r="Z107" t="n">
+        <v>-0.0352</v>
+      </c>
+      <c r="AA107" t="n">
+        <v>-1.59</v>
+      </c>
+      <c r="AB107" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC107" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jimmy Butler III out; Kristaps Porzingis out; Moses Moody out; </t>
+        </is>
+      </c>
+      <c r="AE107" t="inlineStr">
+        <is>
+          <t>over (experimental) (early)</t>
+        </is>
+      </c>
+      <c r="AF107" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>DET @ MIA</t>
+        </is>
+      </c>
+      <c r="C108" t="n">
+        <v>4684742</v>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Ausar Thompson</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>ausar thompson</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>DET</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>MIA</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>AST</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>under</t>
+        </is>
+      </c>
+      <c r="J108" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>fanduel</t>
+        </is>
+      </c>
+      <c r="L108" t="n">
+        <v>-110</v>
+      </c>
+      <c r="M108" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="N108" t="n">
+        <v>0.7246</v>
+      </c>
+      <c r="O108" t="n">
+        <v>0.5373</v>
+      </c>
+      <c r="P108" t="n">
+        <v>0.5681</v>
+      </c>
+      <c r="Q108" t="n">
+        <v>0.0308</v>
+      </c>
+      <c r="R108" t="n">
+        <v>0.08459999999999999</v>
+      </c>
+      <c r="S108" t="n">
+        <v>5.82</v>
+      </c>
+      <c r="T108" t="inlineStr">
+        <is>
+          <t>db951d9ee1d6777d7ced41eba05aac44</t>
+        </is>
+      </c>
+      <c r="U108" t="inlineStr">
+        <is>
+          <t>2026-10-23T12:45:33.160380+00:00</t>
+        </is>
+      </c>
+      <c r="V108" t="n">
+        <v>4</v>
+      </c>
+      <c r="W108" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="X108" t="n">
+        <v>-148</v>
+      </c>
+      <c r="Y108" t="n">
+        <v>0.5639999999999999</v>
+      </c>
+      <c r="Z108" t="n">
+        <v>0.0267</v>
+      </c>
+      <c r="AA108" t="n">
+        <v>5.290909090909092</v>
+      </c>
+      <c r="AB108" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC108" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD108" t="inlineStr"/>
+      <c r="AE108" t="inlineStr">
+        <is>
+          <t>core (early)</t>
+        </is>
+      </c>
+      <c r="AF108" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>NOP @ UTA</t>
+        </is>
+      </c>
+      <c r="C109" t="n">
+        <v>4397688</v>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Trey Murphy III</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>trey murphy</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>NOP</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>UTA</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>PRA</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>over</t>
+        </is>
+      </c>
+      <c r="J109" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>draftkings</t>
+        </is>
+      </c>
+      <c r="L109" t="n">
+        <v>-107</v>
+      </c>
+      <c r="M109" t="n">
+        <v>31.6</v>
+      </c>
+      <c r="N109" t="n">
+        <v>0.6733</v>
+      </c>
+      <c r="O109" t="n">
+        <v>0.4877</v>
+      </c>
+      <c r="P109" t="n">
+        <v>0.5182</v>
+      </c>
+      <c r="Q109" t="n">
+        <v>0.0305</v>
+      </c>
+      <c r="R109" t="n">
+        <v>0.0025</v>
+      </c>
+      <c r="S109" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="T109" t="inlineStr">
+        <is>
+          <t>7469a7f48dbb77001b3148829f80c97b</t>
+        </is>
+      </c>
+      <c r="U109" t="inlineStr">
+        <is>
+          <t>2026-10-23T12:45:33.160380+00:00</t>
+        </is>
+      </c>
+      <c r="V109" t="n">
+        <v>18</v>
+      </c>
+      <c r="W109" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="X109" t="n">
+        <v>-105</v>
+      </c>
+      <c r="Y109" t="n">
+        <v>0.4797</v>
+      </c>
+      <c r="Z109" t="n">
+        <v>-0.008</v>
+      </c>
+      <c r="AA109" t="n">
+        <v>-0.16</v>
+      </c>
+      <c r="AB109" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC109" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD109" t="inlineStr"/>
+      <c r="AE109" t="inlineStr">
+        <is>
+          <t>over (experimental) (early)</t>
+        </is>
+      </c>
+      <c r="AF109" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>DET @ MIA</t>
+        </is>
+      </c>
+      <c r="C110" t="n">
+        <v>3032977</v>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Giannis Antetokounmpo</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>giannis antetokounmpo</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>MIA</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>DET</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>AST</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>under</t>
+        </is>
+      </c>
+      <c r="J110" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>fanduel</t>
+        </is>
+      </c>
+      <c r="L110" t="n">
+        <v>108</v>
+      </c>
+      <c r="M110" t="n">
+        <v>4.96</v>
+      </c>
+      <c r="N110" t="n">
+        <v>0.6254</v>
+      </c>
+      <c r="O110" t="n">
+        <v>0.4596</v>
+      </c>
+      <c r="P110" t="n">
+        <v>0.4844</v>
+      </c>
+      <c r="Q110" t="n">
+        <v>0.0249</v>
+      </c>
+      <c r="R110" t="n">
+        <v>0.0076</v>
+      </c>
+      <c r="S110" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="T110" t="inlineStr">
+        <is>
+          <t>db951d9ee1d6777d7ced41eba05aac44</t>
+        </is>
+      </c>
+      <c r="U110" t="inlineStr">
+        <is>
+          <t>2026-10-23T12:45:33.160380+00:00</t>
+        </is>
+      </c>
+      <c r="V110" t="n">
+        <v>5</v>
+      </c>
+      <c r="W110" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="X110" t="n">
+        <v>110</v>
+      </c>
+      <c r="Y110" t="n">
+        <v>0.4473</v>
+      </c>
+      <c r="Z110" t="n">
+        <v>-0.0123</v>
+      </c>
+      <c r="AA110" t="n">
+        <v>0.9504</v>
+      </c>
+      <c r="AB110" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC110" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD110" t="inlineStr"/>
+      <c r="AE110" t="inlineStr">
+        <is>
+          <t>core (early)</t>
+        </is>
+      </c>
+      <c r="AF110" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>DET @ MIA</t>
+        </is>
+      </c>
+      <c r="C111" t="n">
+        <v>3032977</v>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Giannis Antetokounmpo</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>giannis antetokounmpo</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>MIA</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>DET</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>REB</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>under</t>
+        </is>
+      </c>
+      <c r="J111" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>draftkings</t>
+        </is>
+      </c>
+      <c r="L111" t="n">
+        <v>-117</v>
+      </c>
+      <c r="M111" t="n">
+        <v>9.31</v>
+      </c>
+      <c r="N111" t="n">
+        <v>0.6497000000000001</v>
+      </c>
+      <c r="O111" t="n">
+        <v>0.5226</v>
+      </c>
+      <c r="P111" t="n">
+        <v>0.5417</v>
+      </c>
+      <c r="Q111" t="n">
+        <v>0.0191</v>
+      </c>
+      <c r="R111" t="n">
+        <v>0.0046</v>
+      </c>
+      <c r="S111" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="T111" t="inlineStr">
+        <is>
+          <t>db951d9ee1d6777d7ced41eba05aac44</t>
+        </is>
+      </c>
+      <c r="U111" t="inlineStr">
+        <is>
+          <t>2026-10-23T12:45:33.160380+00:00</t>
+        </is>
+      </c>
+      <c r="V111" t="n">
+        <v>12</v>
+      </c>
+      <c r="W111" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="X111" t="n">
+        <v>-126</v>
+      </c>
+      <c r="Y111" t="n">
+        <v>0.5289</v>
+      </c>
+      <c r="Z111" t="n">
+        <v>0.0063</v>
+      </c>
+      <c r="AA111" t="n">
+        <v>-0.68</v>
+      </c>
+      <c r="AB111" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC111" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD111" t="inlineStr"/>
+      <c r="AE111" t="inlineStr">
+        <is>
+          <t>core (early)</t>
+        </is>
+      </c>
+      <c r="AF111" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Grade picks 2026-10-28: 14 picks from 2026-10-24 graded (6-8, -$20.36)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/performance_report.xlsx
+++ b/outputs/performance_report.xlsx
@@ -474,31 +474,31 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>110</v>
+        <v>124</v>
       </c>
       <c r="C2" t="n">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="D2" t="n">
-        <v>0.464</v>
+        <v>0.46</v>
       </c>
       <c r="E2" t="n">
-        <v>1444.86</v>
+        <v>1490.09</v>
       </c>
       <c r="F2" t="n">
-        <v>-49.92</v>
+        <v>-70.29000000000001</v>
       </c>
       <c r="G2" t="n">
-        <v>-0.0346</v>
+        <v>-0.0472</v>
       </c>
       <c r="H2" t="n">
-        <v>0.542</v>
+        <v>0.539</v>
       </c>
       <c r="I2" t="n">
-        <v>-0.0009</v>
+        <v>-0.0005999999999999999</v>
       </c>
       <c r="J2" t="n">
-        <v>0.455</v>
+        <v>0.427</v>
       </c>
     </row>
   </sheetData>
@@ -574,31 +574,31 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D2" t="n">
-        <v>0.588</v>
+        <v>0.579</v>
       </c>
       <c r="E2" t="n">
-        <v>223.12</v>
+        <v>226.17</v>
       </c>
       <c r="F2" t="n">
-        <v>20.7</v>
+        <v>18.7</v>
       </c>
       <c r="G2" t="n">
-        <v>0.09279999999999999</v>
+        <v>0.0827</v>
       </c>
       <c r="H2" t="n">
-        <v>0.51</v>
+        <v>0.511</v>
       </c>
       <c r="I2" t="n">
-        <v>0.0059</v>
+        <v>0.0016</v>
       </c>
       <c r="J2" t="n">
-        <v>0.588</v>
+        <v>0.526</v>
       </c>
     </row>
     <row r="3">
@@ -608,31 +608,31 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D3" t="n">
-        <v>0.5</v>
+        <v>0.556</v>
       </c>
       <c r="E3" t="n">
-        <v>85.13</v>
+        <v>93.56999999999999</v>
       </c>
       <c r="F3" t="n">
-        <v>14.82</v>
+        <v>21.03</v>
       </c>
       <c r="G3" t="n">
-        <v>0.1741</v>
+        <v>0.2247</v>
       </c>
       <c r="H3" t="n">
-        <v>0.532</v>
+        <v>0.521</v>
       </c>
       <c r="I3" t="n">
         <v>0.0232</v>
       </c>
       <c r="J3" t="n">
-        <v>0.667</v>
+        <v>0.444</v>
       </c>
     </row>
     <row r="4">
@@ -642,22 +642,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C4" t="n">
         <v>21</v>
       </c>
       <c r="D4" t="n">
-        <v>0.42</v>
+        <v>0.404</v>
       </c>
       <c r="E4" t="n">
-        <v>664.1900000000001</v>
+        <v>674.27</v>
       </c>
       <c r="F4" t="n">
-        <v>-70.55</v>
+        <v>-80.63</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.1062</v>
+        <v>-0.1196</v>
       </c>
       <c r="H4" t="n">
         <v>0.551</v>
@@ -666,7 +666,7 @@
         <v>-0.0067</v>
       </c>
       <c r="J4" t="n">
-        <v>0.34</v>
+        <v>0.327</v>
       </c>
     </row>
     <row r="5">
@@ -676,31 +676,31 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C5" t="n">
         <v>12</v>
       </c>
       <c r="D5" t="n">
-        <v>0.545</v>
+        <v>0.5</v>
       </c>
       <c r="E5" t="n">
-        <v>317.62</v>
+        <v>328.92</v>
       </c>
       <c r="F5" t="n">
-        <v>12.33</v>
+        <v>1.03</v>
       </c>
       <c r="G5" t="n">
-        <v>0.0388</v>
+        <v>0.0031</v>
       </c>
       <c r="H5" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.5590000000000001</v>
       </c>
       <c r="I5" t="n">
         <v>-0.008200000000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>0.318</v>
+        <v>0.292</v>
       </c>
     </row>
     <row r="6">
@@ -710,31 +710,31 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C6" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D6" t="n">
-        <v>0.333</v>
+        <v>0.4</v>
       </c>
       <c r="E6" t="n">
-        <v>154.8</v>
+        <v>167.16</v>
       </c>
       <c r="F6" t="n">
-        <v>-27.22</v>
+        <v>-30.41</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.1758</v>
+        <v>-0.1819</v>
       </c>
       <c r="H6" t="n">
-        <v>0.528</v>
+        <v>0.522</v>
       </c>
       <c r="I6" t="n">
-        <v>0.0123</v>
+        <v>0.0163</v>
       </c>
       <c r="J6" t="n">
-        <v>0.8</v>
+        <v>0.75</v>
       </c>
     </row>
   </sheetData>
@@ -810,22 +810,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C2" t="n">
         <v>32</v>
       </c>
       <c r="D2" t="n">
-        <v>0.444</v>
+        <v>0.438</v>
       </c>
       <c r="E2" t="n">
-        <v>947.97</v>
+        <v>949.25</v>
       </c>
       <c r="F2" t="n">
-        <v>-53.5</v>
+        <v>-54.78</v>
       </c>
       <c r="G2" t="n">
-        <v>-0.0564</v>
+        <v>-0.0577</v>
       </c>
       <c r="H2" t="n">
         <v>0.539</v>
@@ -834,7 +834,7 @@
         <v>-0.0068</v>
       </c>
       <c r="J2" t="n">
-        <v>0.347</v>
+        <v>0.342</v>
       </c>
     </row>
     <row r="3">
@@ -844,31 +844,31 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="C3" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="D3" t="n">
-        <v>0.5</v>
+        <v>0.49</v>
       </c>
       <c r="E3" t="n">
-        <v>496.89</v>
+        <v>540.84</v>
       </c>
       <c r="F3" t="n">
-        <v>3.58</v>
+        <v>-15.5</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0072</v>
+        <v>-0.0287</v>
       </c>
       <c r="H3" t="n">
-        <v>0.548</v>
+        <v>0.54</v>
       </c>
       <c r="I3" t="n">
-        <v>0.009900000000000001</v>
+        <v>0.0095</v>
       </c>
       <c r="J3" t="n">
-        <v>0.658</v>
+        <v>0.549</v>
       </c>
     </row>
   </sheetData>
@@ -919,16 +919,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="C2" t="n">
-        <v>0.482</v>
+        <v>0.483</v>
       </c>
       <c r="D2" t="n">
-        <v>0.375</v>
+        <v>0.419</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.107</v>
+        <v>-0.064</v>
       </c>
     </row>
     <row r="3">
@@ -938,16 +938,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C3" t="n">
-        <v>0.537</v>
+        <v>0.536</v>
       </c>
       <c r="D3" t="n">
-        <v>0.5590000000000001</v>
+        <v>0.541</v>
       </c>
       <c r="E3" t="n">
-        <v>0.022</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="4">
@@ -957,16 +957,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C4" t="n">
         <v>0.5610000000000001</v>
       </c>
       <c r="D4" t="n">
-        <v>0.472</v>
+        <v>0.462</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.089</v>
+        <v>-0.099</v>
       </c>
     </row>
     <row r="5">
@@ -976,16 +976,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C5" t="n">
         <v>0.593</v>
       </c>
       <c r="D5" t="n">
-        <v>0.286</v>
+        <v>0.267</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.307</v>
+        <v>-0.326</v>
       </c>
     </row>
     <row r="6">
@@ -1037,7 +1037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF111"/>
+  <dimension ref="A1:AF125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14260,6 +14260,1690 @@
         <v>1</v>
       </c>
     </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>SAS @ DAL</t>
+        </is>
+      </c>
+      <c r="C112" t="n">
+        <v>5037871</v>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Dylan Harper</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>dylan harper</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>SAS</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>DAL</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>PRA</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>under</t>
+        </is>
+      </c>
+      <c r="J112" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>draftkings</t>
+        </is>
+      </c>
+      <c r="L112" t="n">
+        <v>-124</v>
+      </c>
+      <c r="M112" t="n">
+        <v>20.48</v>
+      </c>
+      <c r="N112" t="n">
+        <v>0.8651</v>
+      </c>
+      <c r="O112" t="n">
+        <v>0.5256</v>
+      </c>
+      <c r="P112" t="n">
+        <v>0.585</v>
+      </c>
+      <c r="Q112" t="n">
+        <v>0.0594</v>
+      </c>
+      <c r="R112" t="n">
+        <v>0.0568</v>
+      </c>
+      <c r="S112" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="T112" t="inlineStr">
+        <is>
+          <t>efb2248ad964f84921b3e700125e404b</t>
+        </is>
+      </c>
+      <c r="U112" t="inlineStr">
+        <is>
+          <t>2026-10-24T12:45:39.393320+00:00</t>
+        </is>
+      </c>
+      <c r="V112" t="n">
+        <v>29</v>
+      </c>
+      <c r="W112" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="X112" t="inlineStr"/>
+      <c r="Y112" t="inlineStr"/>
+      <c r="Z112" t="inlineStr"/>
+      <c r="AA112" t="n">
+        <v>-8.800000000000001</v>
+      </c>
+      <c r="AB112" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC112" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tobias Harris out; </t>
+        </is>
+      </c>
+      <c r="AE112" t="inlineStr">
+        <is>
+          <t>blowout (early)</t>
+        </is>
+      </c>
+      <c r="AF112" t="n">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>SAS @ DAL</t>
+        </is>
+      </c>
+      <c r="C113" t="n">
+        <v>5037871</v>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Dylan Harper</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>dylan harper</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>SAS</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>DAL</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>PTS</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>under</t>
+        </is>
+      </c>
+      <c r="J113" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>williamhill_us</t>
+        </is>
+      </c>
+      <c r="L113" t="n">
+        <v>-124</v>
+      </c>
+      <c r="M113" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="N113" t="n">
+        <v>0.8369</v>
+      </c>
+      <c r="O113" t="n">
+        <v>0.5237000000000001</v>
+      </c>
+      <c r="P113" t="n">
+        <v>0.5785</v>
+      </c>
+      <c r="Q113" t="n">
+        <v>0.0548</v>
+      </c>
+      <c r="R113" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="S113" t="n">
+        <v>6.98</v>
+      </c>
+      <c r="T113" t="inlineStr">
+        <is>
+          <t>efb2248ad964f84921b3e700125e404b</t>
+        </is>
+      </c>
+      <c r="U113" t="inlineStr">
+        <is>
+          <t>2026-10-24T12:45:39.393320+00:00</t>
+        </is>
+      </c>
+      <c r="V113" t="n">
+        <v>22</v>
+      </c>
+      <c r="W113" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="X113" t="inlineStr"/>
+      <c r="Y113" t="inlineStr"/>
+      <c r="Z113" t="inlineStr"/>
+      <c r="AA113" t="n">
+        <v>-6.98</v>
+      </c>
+      <c r="AB113" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC113" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tobias Harris out; </t>
+        </is>
+      </c>
+      <c r="AE113" t="inlineStr">
+        <is>
+          <t>blowout (early)</t>
+        </is>
+      </c>
+      <c r="AF113" t="n">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>WAS @ CHI</t>
+        </is>
+      </c>
+      <c r="C114" t="n">
+        <v>5160992</v>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Alex Sarr</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>alex sarr</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>WAS</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>CHI</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>PRA</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>over</t>
+        </is>
+      </c>
+      <c r="J114" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>betrivers</t>
+        </is>
+      </c>
+      <c r="L114" t="n">
+        <v>-105</v>
+      </c>
+      <c r="M114" t="n">
+        <v>25.29</v>
+      </c>
+      <c r="N114" t="n">
+        <v>0.6921</v>
+      </c>
+      <c r="O114" t="n">
+        <v>0.4861</v>
+      </c>
+      <c r="P114" t="n">
+        <v>0.5222</v>
+      </c>
+      <c r="Q114" t="n">
+        <v>0.036</v>
+      </c>
+      <c r="R114" t="n">
+        <v>0.0195</v>
+      </c>
+      <c r="S114" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="T114" t="inlineStr">
+        <is>
+          <t>cce3cd5869541979d68f7bde648f7c20</t>
+        </is>
+      </c>
+      <c r="U114" t="inlineStr">
+        <is>
+          <t>2026-10-24T12:45:39.393320+00:00</t>
+        </is>
+      </c>
+      <c r="V114" t="n">
+        <v>15</v>
+      </c>
+      <c r="W114" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="X114" t="inlineStr"/>
+      <c r="Y114" t="inlineStr"/>
+      <c r="Z114" t="inlineStr"/>
+      <c r="AA114" t="n">
+        <v>-1.28</v>
+      </c>
+      <c r="AB114" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC114" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jamir Watkins out; Tristan Vukcevic out; </t>
+        </is>
+      </c>
+      <c r="AE114" t="inlineStr">
+        <is>
+          <t>over (experimental) (early)</t>
+        </is>
+      </c>
+      <c r="AF114" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>MIA @ CHA</t>
+        </is>
+      </c>
+      <c r="C115" t="n">
+        <v>3032977</v>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Giannis Antetokounmpo</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>giannis antetokounmpo</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>MIA</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>CHA</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>REB</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>under</t>
+        </is>
+      </c>
+      <c r="J115" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>fanduel</t>
+        </is>
+      </c>
+      <c r="L115" t="n">
+        <v>108</v>
+      </c>
+      <c r="M115" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="N115" t="n">
+        <v>0.6793</v>
+      </c>
+      <c r="O115" t="n">
+        <v>0.4558</v>
+      </c>
+      <c r="P115" t="n">
+        <v>0.4893</v>
+      </c>
+      <c r="Q115" t="n">
+        <v>0.0335</v>
+      </c>
+      <c r="R115" t="n">
+        <v>0.0178</v>
+      </c>
+      <c r="S115" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="T115" t="inlineStr">
+        <is>
+          <t>0abd50d04d02296b33809f9458fd47e4</t>
+        </is>
+      </c>
+      <c r="U115" t="inlineStr">
+        <is>
+          <t>2026-10-24T12:45:39.393320+00:00</t>
+        </is>
+      </c>
+      <c r="V115" t="n">
+        <v>6</v>
+      </c>
+      <c r="W115" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="X115" t="n">
+        <v>-120</v>
+      </c>
+      <c r="Y115" t="n">
+        <v>0.4921</v>
+      </c>
+      <c r="Z115" t="n">
+        <v>0.0363</v>
+      </c>
+      <c r="AA115" t="n">
+        <v>2.2248</v>
+      </c>
+      <c r="AB115" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC115" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD115" t="inlineStr"/>
+      <c r="AE115" t="inlineStr">
+        <is>
+          <t>core (early)</t>
+        </is>
+      </c>
+      <c r="AF115" t="n">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>SAS @ DAL</t>
+        </is>
+      </c>
+      <c r="C116" t="n">
+        <v>5037871</v>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Dylan Harper</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>dylan harper</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>SAS</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>DAL</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>REB</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>under</t>
+        </is>
+      </c>
+      <c r="J116" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>betmgm</t>
+        </is>
+      </c>
+      <c r="L116" t="n">
+        <v>-105</v>
+      </c>
+      <c r="M116" t="n">
+        <v>3.72</v>
+      </c>
+      <c r="N116" t="n">
+        <v>0.6834</v>
+      </c>
+      <c r="O116" t="n">
+        <v>0.4985</v>
+      </c>
+      <c r="P116" t="n">
+        <v>0.5308</v>
+      </c>
+      <c r="Q116" t="n">
+        <v>0.0324</v>
+      </c>
+      <c r="R116" t="n">
+        <v>0.0363</v>
+      </c>
+      <c r="S116" t="n">
+        <v>4.77</v>
+      </c>
+      <c r="T116" t="inlineStr">
+        <is>
+          <t>efb2248ad964f84921b3e700125e404b</t>
+        </is>
+      </c>
+      <c r="U116" t="inlineStr">
+        <is>
+          <t>2026-10-24T12:45:39.393320+00:00</t>
+        </is>
+      </c>
+      <c r="V116" t="n">
+        <v>5</v>
+      </c>
+      <c r="W116" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="X116" t="inlineStr"/>
+      <c r="Y116" t="inlineStr"/>
+      <c r="Z116" t="inlineStr"/>
+      <c r="AA116" t="n">
+        <v>-4.77</v>
+      </c>
+      <c r="AB116" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC116" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tobias Harris out; </t>
+        </is>
+      </c>
+      <c r="AE116" t="inlineStr">
+        <is>
+          <t>blowout (early)</t>
+        </is>
+      </c>
+      <c r="AF116" t="n">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>NOP @ DEN</t>
+        </is>
+      </c>
+      <c r="C117" t="n">
+        <v>4431767</v>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Christian Braun</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>christian braun</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>DEN</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>NOP</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>FG3M</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>under</t>
+        </is>
+      </c>
+      <c r="J117" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>betmgm</t>
+        </is>
+      </c>
+      <c r="L117" t="n">
+        <v>-110</v>
+      </c>
+      <c r="M117" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="N117" t="n">
+        <v>0.7108</v>
+      </c>
+      <c r="O117" t="n">
+        <v>0.5198</v>
+      </c>
+      <c r="P117" t="n">
+        <v>0.5512</v>
+      </c>
+      <c r="Q117" t="n">
+        <v>0.0314</v>
+      </c>
+      <c r="R117" t="n">
+        <v>0.0522</v>
+      </c>
+      <c r="S117" t="n">
+        <v>7.18</v>
+      </c>
+      <c r="T117" t="inlineStr">
+        <is>
+          <t>0c95f2515a34d871cd4946cbf38dd670</t>
+        </is>
+      </c>
+      <c r="U117" t="inlineStr">
+        <is>
+          <t>2026-10-24T12:45:39.393320+00:00</t>
+        </is>
+      </c>
+      <c r="V117" t="n">
+        <v>0</v>
+      </c>
+      <c r="W117" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="X117" t="inlineStr"/>
+      <c r="Y117" t="inlineStr"/>
+      <c r="Z117" t="inlineStr"/>
+      <c r="AA117" t="n">
+        <v>6.527272727272727</v>
+      </c>
+      <c r="AB117" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC117" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cameron Johnson out; Julian Strawther out; Spencer Jones out; </t>
+        </is>
+      </c>
+      <c r="AE117" t="inlineStr">
+        <is>
+          <t>blowout (early)</t>
+        </is>
+      </c>
+      <c r="AF117" t="n">
+        <v>11.5</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>MIA @ CHA</t>
+        </is>
+      </c>
+      <c r="C118" t="n">
+        <v>3032977</v>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Giannis Antetokounmpo</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>giannis antetokounmpo</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>MIA</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>CHA</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>AST</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>under</t>
+        </is>
+      </c>
+      <c r="J118" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>fanatics</t>
+        </is>
+      </c>
+      <c r="L118" t="n">
+        <v>105</v>
+      </c>
+      <c r="M118" t="n">
+        <v>5.01</v>
+      </c>
+      <c r="N118" t="n">
+        <v>0.6175</v>
+      </c>
+      <c r="O118" t="n">
+        <v>0.4674</v>
+      </c>
+      <c r="P118" t="n">
+        <v>0.4899</v>
+      </c>
+      <c r="Q118" t="n">
+        <v>0.0225</v>
+      </c>
+      <c r="R118" t="n">
+        <v>0.0043</v>
+      </c>
+      <c r="S118" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="T118" t="inlineStr">
+        <is>
+          <t>0abd50d04d02296b33809f9458fd47e4</t>
+        </is>
+      </c>
+      <c r="U118" t="inlineStr">
+        <is>
+          <t>2026-10-24T12:45:39.393320+00:00</t>
+        </is>
+      </c>
+      <c r="V118" t="n">
+        <v>3</v>
+      </c>
+      <c r="W118" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="X118" t="inlineStr"/>
+      <c r="Y118" t="n">
+        <v>0.4085</v>
+      </c>
+      <c r="Z118" t="n">
+        <v>-0.0589</v>
+      </c>
+      <c r="AA118" t="n">
+        <v>0.5354999999999999</v>
+      </c>
+      <c r="AB118" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC118" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD118" t="inlineStr"/>
+      <c r="AE118" t="inlineStr">
+        <is>
+          <t>core (early)</t>
+        </is>
+      </c>
+      <c r="AF118" t="n">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>MIA @ CHA</t>
+        </is>
+      </c>
+      <c r="C119" t="n">
+        <v>4066261</v>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Bam Adebayo</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>bam adebayo</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>MIA</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>CHA</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>REB</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>under</t>
+        </is>
+      </c>
+      <c r="J119" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>betmgm</t>
+        </is>
+      </c>
+      <c r="L119" t="n">
+        <v>-111</v>
+      </c>
+      <c r="M119" t="n">
+        <v>8.56</v>
+      </c>
+      <c r="N119" t="n">
+        <v>0.6354</v>
+      </c>
+      <c r="O119" t="n">
+        <v>0.5123</v>
+      </c>
+      <c r="P119" t="n">
+        <v>0.5339</v>
+      </c>
+      <c r="Q119" t="n">
+        <v>0.0215</v>
+      </c>
+      <c r="R119" t="n">
+        <v>0.0148</v>
+      </c>
+      <c r="S119" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="T119" t="inlineStr">
+        <is>
+          <t>0abd50d04d02296b33809f9458fd47e4</t>
+        </is>
+      </c>
+      <c r="U119" t="inlineStr">
+        <is>
+          <t>2026-10-24T12:45:39.393320+00:00</t>
+        </is>
+      </c>
+      <c r="V119" t="n">
+        <v>8</v>
+      </c>
+      <c r="W119" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="X119" t="n">
+        <v>-125</v>
+      </c>
+      <c r="Y119" t="n">
+        <v>0.5527</v>
+      </c>
+      <c r="Z119" t="n">
+        <v>0.0404</v>
+      </c>
+      <c r="AA119" t="n">
+        <v>1.855855855855856</v>
+      </c>
+      <c r="AB119" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC119" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD119" t="inlineStr"/>
+      <c r="AE119" t="inlineStr">
+        <is>
+          <t>core (early)</t>
+        </is>
+      </c>
+      <c r="AF119" t="n">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>MIA @ CHA</t>
+        </is>
+      </c>
+      <c r="C120" t="n">
+        <v>4278053</v>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Davion Mitchell</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>davion mitchell</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>MIA</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>CHA</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>REB</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>under</t>
+        </is>
+      </c>
+      <c r="J120" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>fanduel</t>
+        </is>
+      </c>
+      <c r="L120" t="n">
+        <v>116</v>
+      </c>
+      <c r="M120" t="n">
+        <v>2.42</v>
+      </c>
+      <c r="N120" t="n">
+        <v>0.5645</v>
+      </c>
+      <c r="O120" t="n">
+        <v>0.4438</v>
+      </c>
+      <c r="P120" t="n">
+        <v>0.4649</v>
+      </c>
+      <c r="Q120" t="n">
+        <v>0.0211</v>
+      </c>
+      <c r="R120" t="n">
+        <v>0.0042</v>
+      </c>
+      <c r="S120" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="T120" t="inlineStr">
+        <is>
+          <t>0abd50d04d02296b33809f9458fd47e4</t>
+        </is>
+      </c>
+      <c r="U120" t="inlineStr">
+        <is>
+          <t>2026-10-24T12:45:39.393320+00:00</t>
+        </is>
+      </c>
+      <c r="V120" t="n">
+        <v>1</v>
+      </c>
+      <c r="W120" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="X120" t="n">
+        <v>-120</v>
+      </c>
+      <c r="Y120" t="n">
+        <v>0.4724</v>
+      </c>
+      <c r="Z120" t="n">
+        <v>0.0286</v>
+      </c>
+      <c r="AA120" t="n">
+        <v>0.5220000000000001</v>
+      </c>
+      <c r="AB120" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC120" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD120" t="inlineStr"/>
+      <c r="AE120" t="inlineStr">
+        <is>
+          <t>core (early)</t>
+        </is>
+      </c>
+      <c r="AF120" t="n">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>MIA @ CHA</t>
+        </is>
+      </c>
+      <c r="C121" t="n">
+        <v>4066261</v>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Bam Adebayo</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>bam adebayo</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>MIA</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>CHA</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>AST</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>under</t>
+        </is>
+      </c>
+      <c r="J121" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>williamhill_us</t>
+        </is>
+      </c>
+      <c r="L121" t="n">
+        <v>-118</v>
+      </c>
+      <c r="M121" t="n">
+        <v>3.02</v>
+      </c>
+      <c r="N121" t="n">
+        <v>0.6449</v>
+      </c>
+      <c r="O121" t="n">
+        <v>0.5306</v>
+      </c>
+      <c r="P121" t="n">
+        <v>0.5506</v>
+      </c>
+      <c r="Q121" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="R121" t="n">
+        <v>0.0172</v>
+      </c>
+      <c r="S121" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="T121" t="inlineStr">
+        <is>
+          <t>0abd50d04d02296b33809f9458fd47e4</t>
+        </is>
+      </c>
+      <c r="U121" t="inlineStr">
+        <is>
+          <t>2026-10-24T12:45:39.393320+00:00</t>
+        </is>
+      </c>
+      <c r="V121" t="n">
+        <v>4</v>
+      </c>
+      <c r="W121" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="X121" t="n">
+        <v>-125</v>
+      </c>
+      <c r="Y121" t="n">
+        <v>0.5188</v>
+      </c>
+      <c r="Z121" t="n">
+        <v>-0.0118</v>
+      </c>
+      <c r="AA121" t="n">
+        <v>-2.54</v>
+      </c>
+      <c r="AB121" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC121" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD121" t="inlineStr"/>
+      <c r="AE121" t="inlineStr">
+        <is>
+          <t>core (early)</t>
+        </is>
+      </c>
+      <c r="AF121" t="n">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>MIL @ PHI</t>
+        </is>
+      </c>
+      <c r="C122" t="n">
+        <v>3059318</v>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Joel Embiid</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>joel embiid</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>MIL</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>REB</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>under</t>
+        </is>
+      </c>
+      <c r="J122" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>betmgm</t>
+        </is>
+      </c>
+      <c r="L122" t="n">
+        <v>105</v>
+      </c>
+      <c r="M122" t="n">
+        <v>7.99</v>
+      </c>
+      <c r="N122" t="n">
+        <v>0.5939</v>
+      </c>
+      <c r="O122" t="n">
+        <v>0.4803</v>
+      </c>
+      <c r="P122" t="n">
+        <v>0.5002</v>
+      </c>
+      <c r="Q122" t="n">
+        <v>0.0199</v>
+      </c>
+      <c r="R122" t="n">
+        <v>0.0254</v>
+      </c>
+      <c r="S122" t="n">
+        <v>3.02</v>
+      </c>
+      <c r="T122" t="inlineStr">
+        <is>
+          <t>a66da208d3609b028970dfe2b5d7973f</t>
+        </is>
+      </c>
+      <c r="U122" t="inlineStr">
+        <is>
+          <t>2026-10-24T12:45:39.393320+00:00</t>
+        </is>
+      </c>
+      <c r="V122" t="n">
+        <v>11</v>
+      </c>
+      <c r="W122" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="X122" t="inlineStr"/>
+      <c r="Y122" t="inlineStr"/>
+      <c r="Z122" t="inlineStr"/>
+      <c r="AA122" t="n">
+        <v>-3.02</v>
+      </c>
+      <c r="AB122" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC122" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD122" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LeBron James out; Dominick Barlow out; Ariel Hukporti out; </t>
+        </is>
+      </c>
+      <c r="AE122" t="inlineStr">
+        <is>
+          <t>blowout (early)</t>
+        </is>
+      </c>
+      <c r="AF122" t="n">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>BKN @ CLE</t>
+        </is>
+      </c>
+      <c r="C123" t="n">
+        <v>5175643</v>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Egor Demin</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>egor demin</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>BKN</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>CLE</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>PTS</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>under</t>
+        </is>
+      </c>
+      <c r="J123" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>williamhill_us</t>
+        </is>
+      </c>
+      <c r="L123" t="n">
+        <v>105</v>
+      </c>
+      <c r="M123" t="n">
+        <v>10</v>
+      </c>
+      <c r="N123" t="n">
+        <v>0.6056</v>
+      </c>
+      <c r="O123" t="n">
+        <v>0.4858</v>
+      </c>
+      <c r="P123" t="n">
+        <v>0.5054999999999999</v>
+      </c>
+      <c r="Q123" t="n">
+        <v>0.0197</v>
+      </c>
+      <c r="R123" t="n">
+        <v>0.0363</v>
+      </c>
+      <c r="S123" t="n">
+        <v>4.32</v>
+      </c>
+      <c r="T123" t="inlineStr">
+        <is>
+          <t>f187c8a86c1d1676bb45b9b3a6707872</t>
+        </is>
+      </c>
+      <c r="U123" t="inlineStr">
+        <is>
+          <t>2026-10-24T12:45:39.393320+00:00</t>
+        </is>
+      </c>
+      <c r="V123" t="n">
+        <v>22</v>
+      </c>
+      <c r="W123" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="X123" t="inlineStr"/>
+      <c r="Y123" t="inlineStr"/>
+      <c r="Z123" t="inlineStr"/>
+      <c r="AA123" t="n">
+        <v>-4.32</v>
+      </c>
+      <c r="AB123" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC123" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD123" t="inlineStr"/>
+      <c r="AE123" t="inlineStr">
+        <is>
+          <t>blowout (early)</t>
+        </is>
+      </c>
+      <c r="AF123" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>MIL @ PHI</t>
+        </is>
+      </c>
+      <c r="C124" t="n">
+        <v>3059318</v>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Joel Embiid</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>joel embiid</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>MIL</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>FG3M</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>under</t>
+        </is>
+      </c>
+      <c r="J124" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>draftkings</t>
+        </is>
+      </c>
+      <c r="L124" t="n">
+        <v>-104</v>
+      </c>
+      <c r="M124" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="N124" t="n">
+        <v>0.5953000000000001</v>
+      </c>
+      <c r="O124" t="n">
+        <v>0.4939</v>
+      </c>
+      <c r="P124" t="n">
+        <v>0.5117</v>
+      </c>
+      <c r="Q124" t="n">
+        <v>0.0177</v>
+      </c>
+      <c r="R124" t="n">
+        <v>0.0037</v>
+      </c>
+      <c r="S124" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="T124" t="inlineStr">
+        <is>
+          <t>a66da208d3609b028970dfe2b5d7973f</t>
+        </is>
+      </c>
+      <c r="U124" t="inlineStr">
+        <is>
+          <t>2026-10-24T12:45:39.393320+00:00</t>
+        </is>
+      </c>
+      <c r="V124" t="n">
+        <v>0</v>
+      </c>
+      <c r="W124" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="X124" t="inlineStr"/>
+      <c r="Y124" t="inlineStr"/>
+      <c r="Z124" t="inlineStr"/>
+      <c r="AA124" t="n">
+        <v>0.4615384615384616</v>
+      </c>
+      <c r="AB124" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC124" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD124" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LeBron James out; Dominick Barlow out; Ariel Hukporti out; </t>
+        </is>
+      </c>
+      <c r="AE124" t="inlineStr">
+        <is>
+          <t>blowout (early)</t>
+        </is>
+      </c>
+      <c r="AF124" t="n">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>SAS @ DAL</t>
+        </is>
+      </c>
+      <c r="C125" t="n">
+        <v>5104157</v>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Victor Wembanyama</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>victor wembanyama</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>SAS</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>DAL</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>FG3M</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>under</t>
+        </is>
+      </c>
+      <c r="J125" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>betmgm</t>
+        </is>
+      </c>
+      <c r="L125" t="n">
+        <v>130</v>
+      </c>
+      <c r="M125" t="n">
+        <v>1.82</v>
+      </c>
+      <c r="N125" t="n">
+        <v>0.5124</v>
+      </c>
+      <c r="O125" t="n">
+        <v>0.4226</v>
+      </c>
+      <c r="P125" t="n">
+        <v>0.4383</v>
+      </c>
+      <c r="Q125" t="n">
+        <v>0.0157</v>
+      </c>
+      <c r="R125" t="n">
+        <v>0.008</v>
+      </c>
+      <c r="S125" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="T125" t="inlineStr">
+        <is>
+          <t>efb2248ad964f84921b3e700125e404b</t>
+        </is>
+      </c>
+      <c r="U125" t="inlineStr">
+        <is>
+          <t>2026-10-24T12:45:39.393320+00:00</t>
+        </is>
+      </c>
+      <c r="V125" t="n">
+        <v>2</v>
+      </c>
+      <c r="W125" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="X125" t="inlineStr"/>
+      <c r="Y125" t="inlineStr"/>
+      <c r="Z125" t="inlineStr"/>
+      <c r="AA125" t="n">
+        <v>-0.78</v>
+      </c>
+      <c r="AB125" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC125" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD125" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tobias Harris out; </t>
+        </is>
+      </c>
+      <c r="AE125" t="inlineStr">
+        <is>
+          <t>blowout (early)</t>
+        </is>
+      </c>
+      <c r="AF125" t="n">
+        <v>12.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>